<commit_message>
Add recorded Malayalam clips, English clip list and English support in the clip generator
- 82 Malayalam clips generated with ElevenLabs (77 are used; 5 belong to questions the app never asks)
- npm run tts -- --lang en: English list with rupees, A plus and Plus Two spelt out for speech; separate voice via ELEVENLABS_VOICE_ID_EN
- Plainer English questions (person applying, your family, BPL spelt out); English ranges read "23 to 59 years", "5 years or more", "1 year"
</commit_message>
<xml_diff>
--- a/dataset/anavandi-dataset.xlsx
+++ b/dataset/anavandi-dataset.xlsx
@@ -9132,8 +9132,6 @@
           <t>PLNT-04=potentially_eligible</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>AI-review</t>
@@ -9171,8 +9169,6 @@
           <t>PLNT-04=not_matched</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>AI-review</t>
@@ -9210,8 +9206,6 @@
           <t>PLNT-01=not_matched</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>AI-review</t>
@@ -9249,8 +9243,6 @@
           <t>PLNT-06=potentially_eligible; PLNT-07=potentially_eligible</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>AI-review</t>
@@ -9288,8 +9280,6 @@
           <t>PLNT-06=potentially_eligible; PLNT-07=not_matched</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>AI-review</t>
@@ -9327,7 +9317,6 @@
           <t>PLNT-09=potentially_eligible; PLNT-08=needs_information</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>PLNT-08:plantation_child_class10</t>
@@ -9370,8 +9359,6 @@
           <t>PLNT-02=not_matched</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>AI-review</t>
@@ -9409,8 +9396,6 @@
           <t>FISH-21=potentially_eligible; FISH-16=not_matched; FISH-22=not_matched</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>AI-review</t>
@@ -9448,8 +9433,6 @@
           <t>FISH-21=not_matched</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>AI-review</t>
@@ -9487,8 +9470,6 @@
           <t>FISH-22=potentially_eligible; FISH-16=not_matched; FISH-21=not_matched</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>AI-review</t>
@@ -11597,7 +11578,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Which work does your household do?</t>
+          <t>What work does your family do?</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -11647,7 +11628,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Is the beneficiary a registered fisherman?</t>
+          <t>Is the person applying a registered fisher?</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -11697,7 +11678,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Is the beneficiary an active fisherman?</t>
+          <t>Does the person applying still work as a fisher (an active fisher)?</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -11737,7 +11718,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Is the household in the BPL category?</t>
+          <t>Is your family in the BPL (below poverty line) category?</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -11777,7 +11758,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Does the beneficiary have a bank account?</t>
+          <t>Does the person applying have a bank account?</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -11817,7 +11798,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Is the beneficiary a registered traditional fisherman?</t>
+          <t>Is the person applying a registered traditional fisher?</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -12457,7 +12438,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Has the person stopped (retired from) fishing work?</t>
+          <t>Has the person stopped fishing work (retired)?</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -12497,7 +12478,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>What is the family's total income in a year?</t>
+          <t>What is your family's total income in a year?</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">

</xml_diff>